<commit_message>
match test case to full case
</commit_message>
<xml_diff>
--- a/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_all_configs.xlsx
+++ b/test_data/norfolk_coastal_flooding/full_benchmarking_experiment_uva_test_all_configs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\dcl3nd\dev\TRITON-SWMM_toolkit\test_data\norfolk_coastal_flooding\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E925DD9-5641-42C4-82B6-8306B7F27853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{843E6565-3387-41E0-8784-C5F031409B05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="19">
   <si>
     <t>run_mode</t>
   </si>
@@ -88,6 +88,9 @@
   <si>
     <t>gpu</t>
   </si>
+  <si>
+    <t>gpu-a6000</t>
+  </si>
 </sst>
 </file>
 
@@ -127,7 +130,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -142,12 +145,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -223,14 +220,16 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FFC6C6C6"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -268,26 +267,14 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="3" fontId="3" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="7">
     <dxf>
       <font>
         <b val="0"/>
@@ -329,6 +316,256 @@
         <horizontal/>
       </border>
     </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="3" formatCode="#,##0"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF3F3F76"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFFFCC99"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color rgb="FF000000"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF000000"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF000000"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF000000"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -343,18 +580,18 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K28" totalsRowShown="0">
-  <autoFilter ref="A1:K28" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K38" totalsRowShown="0">
+  <autoFilter ref="A1:K38" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K21">
     <sortCondition ref="I1:I23"/>
   </sortState>
   <tableColumns count="11">
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode"/>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="n_nodes"/>
-    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="n_mpi_procs"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="n_omp_threads"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n_gpus"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="hpc_ensemble_partition"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="run_mode" dataDxfId="6"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="n_nodes" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="n_mpi_procs" dataDxfId="4"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="n_omp_threads" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="n_gpus" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="hpc_ensemble_partition" dataDxfId="1"/>
     <tableColumn id="9" xr3:uid="{26339B98-C3B5-4C3B-9409-F4B744B2B94C}" name="mem_gb_per_cpu" dataDxfId="0"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="total_OpenMP_threads"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="total_devices"/>
@@ -653,7 +890,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.28515625" style="11" bestFit="1" customWidth="1"/>
@@ -705,7 +942,7 @@
     </row>
     <row r="2" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B2" s="7">
         <v>1</v>
@@ -717,13 +954,13 @@
         <v>1</v>
       </c>
       <c r="E2" s="7">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G2" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H2" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
@@ -744,25 +981,25 @@
     </row>
     <row r="3" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B3" s="7">
         <v>1</v>
       </c>
       <c r="C3" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D3" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F3" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G3" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H3" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
@@ -783,37 +1020,37 @@
     </row>
     <row r="4" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B4" s="7">
         <v>1</v>
       </c>
       <c r="C4" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D4" s="7">
         <v>1</v>
       </c>
       <c r="E4" s="7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G4" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H4" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J4" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K4" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -822,25 +1059,25 @@
     </row>
     <row r="5" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5" s="7">
         <v>1</v>
       </c>
       <c r="C5" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D5" s="7">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E5" s="7">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G5" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H5" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
@@ -861,37 +1098,37 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B6" s="7">
         <v>1</v>
       </c>
       <c r="C6" s="7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="7">
         <v>1</v>
       </c>
       <c r="E6" s="7">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F6" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G6" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H6" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="I6" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -900,37 +1137,37 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="B7" s="7">
         <v>1</v>
       </c>
       <c r="C7" s="7">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D7" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E7" s="7">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G7" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H7" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="I7" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="J7" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K7" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -939,37 +1176,37 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B8" s="7">
         <v>1</v>
       </c>
       <c r="C8" s="7">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D8" s="7">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E8" s="7">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F8" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G8" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H8" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="I8" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="J8" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K8" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -978,7 +1215,7 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B9" s="7">
         <v>1</v>
@@ -990,13 +1227,13 @@
         <v>1</v>
       </c>
       <c r="E9" s="7">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F9" s="8" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="G9" s="8">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="H9" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
@@ -1026,7 +1263,7 @@
         <v>2</v>
       </c>
       <c r="D10" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E10" s="7">
         <v>0</v>
@@ -1039,15 +1276,15 @@
       </c>
       <c r="H10" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="I10" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="J10" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K10" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1056,16 +1293,16 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="B11" s="7">
+        <v>9</v>
+      </c>
+      <c r="B11" s="13">
         <v>1</v>
       </c>
       <c r="C11" s="7">
-        <v>16</v>
-      </c>
-      <c r="D11" s="7">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="D11" s="13">
+        <v>4</v>
       </c>
       <c r="E11" s="7">
         <v>0</v>
@@ -1078,15 +1315,15 @@
       </c>
       <c r="H11" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I11" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J11" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K11" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1101,10 +1338,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D12" s="7">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E12" s="7">
         <v>0</v>
@@ -1112,20 +1349,20 @@
       <c r="F12" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G12" s="13">
+      <c r="G12" s="8">
         <v>2</v>
       </c>
       <c r="H12" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="I12" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="J12" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="K12" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1134,16 +1371,16 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B13" s="7">
         <v>1</v>
       </c>
       <c r="C13" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" s="7">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="E13" s="7">
         <v>0</v>
@@ -1173,16 +1410,16 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B14" s="7">
         <v>1</v>
       </c>
       <c r="C14" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D14" s="7">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="E14" s="7">
         <v>0</v>
@@ -1195,15 +1432,15 @@
       </c>
       <c r="H14" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="I14" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="J14" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="K14" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1218,10 +1455,10 @@
         <v>1</v>
       </c>
       <c r="C15" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D15" s="7">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="E15" s="7">
         <v>0</v>
@@ -1234,15 +1471,15 @@
       </c>
       <c r="H15" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="I15" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="J15" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="K15" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1257,31 +1494,31 @@
         <v>1</v>
       </c>
       <c r="C16" s="7">
+        <v>2</v>
+      </c>
+      <c r="D16" s="7">
+        <v>16</v>
+      </c>
+      <c r="E16" s="7">
+        <v>0</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G16" s="8">
+        <v>2</v>
+      </c>
+      <c r="H16" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="D16" s="7">
-        <v>2</v>
-      </c>
-      <c r="E16" s="7">
-        <v>0</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G16" s="8">
-        <v>2</v>
-      </c>
-      <c r="H16" s="9">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
-      </c>
       <c r="I16" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="J16" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="K16" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1290,16 +1527,16 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B17" s="7">
         <v>1</v>
       </c>
       <c r="C17" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D17" s="7">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="E17" s="7">
         <v>0</v>
@@ -1312,15 +1549,15 @@
       </c>
       <c r="H17" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="I17" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="J17" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="K17" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1335,31 +1572,31 @@
         <v>1</v>
       </c>
       <c r="C18" s="7">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D18" s="7">
+        <v>4</v>
+      </c>
+      <c r="E18" s="7">
+        <v>0</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G18" s="8">
+        <v>2</v>
+      </c>
+      <c r="H18" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="E18" s="7">
-        <v>0</v>
-      </c>
-      <c r="F18" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G18" s="8">
-        <v>2</v>
-      </c>
-      <c r="H18" s="9">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>64</v>
-      </c>
       <c r="I18" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="J18" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="K18" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1371,34 +1608,34 @@
         <v>9</v>
       </c>
       <c r="B19" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C19" s="7">
+        <v>16</v>
+      </c>
+      <c r="D19" s="7">
+        <v>2</v>
+      </c>
+      <c r="E19" s="7">
+        <v>0</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G19" s="8">
+        <v>2</v>
+      </c>
+      <c r="H19" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>32</v>
       </c>
-      <c r="D19" s="7">
-        <v>4</v>
-      </c>
-      <c r="E19" s="7">
-        <v>0</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="8">
-        <v>2</v>
-      </c>
-      <c r="H19" s="9">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
-      </c>
       <c r="I19" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>32</v>
       </c>
       <c r="J19" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="K19" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1410,30 +1647,30 @@
         <v>9</v>
       </c>
       <c r="B20" s="7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C20" s="7">
+        <v>2</v>
+      </c>
+      <c r="D20" s="7">
+        <v>32</v>
+      </c>
+      <c r="E20" s="7">
+        <v>0</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G20" s="8">
+        <v>2</v>
+      </c>
+      <c r="H20" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="D20" s="7">
-        <v>2</v>
-      </c>
-      <c r="E20" s="7">
-        <v>0</v>
-      </c>
-      <c r="F20" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="8">
-        <v>2</v>
-      </c>
-      <c r="H20" s="9">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
-      </c>
       <c r="I20" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="J20" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
@@ -1452,31 +1689,31 @@
         <v>1</v>
       </c>
       <c r="C21" s="7">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D21" s="7">
+        <v>16</v>
+      </c>
+      <c r="E21" s="7">
+        <v>0</v>
+      </c>
+      <c r="F21" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G21" s="8">
+        <v>2</v>
+      </c>
+      <c r="H21" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
         <v>64</v>
       </c>
-      <c r="E21" s="7">
-        <v>0</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G21" s="8">
-        <v>2</v>
-      </c>
-      <c r="H21" s="9">
-        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>128</v>
-      </c>
       <c r="I21" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="J21" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>128</v>
+        <v>64</v>
       </c>
       <c r="K21" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1485,37 +1722,37 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B22" s="7">
         <v>1</v>
       </c>
       <c r="C22" s="7">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="D22" s="7">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E22" s="7">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G22" s="13">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="G22" s="8">
+        <v>2</v>
       </c>
       <c r="H22" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="I22" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="J22" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="K22" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1524,37 +1761,37 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B23" s="7">
         <v>1</v>
       </c>
       <c r="C23" s="7">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D23" s="7">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E23" s="7">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G23" s="13">
-        <v>8</v>
+        <v>10</v>
+      </c>
+      <c r="G23" s="8">
+        <v>2</v>
       </c>
       <c r="H23" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="I23" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="J23" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="K23" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1563,37 +1800,37 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B24" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C24" s="7">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D24" s="7">
-        <v>1</v>
+        <v>64</v>
       </c>
       <c r="E24" s="7">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G24" s="13">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="G24" s="8">
+        <v>2</v>
       </c>
       <c r="H24" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>5</v>
+        <v>128</v>
       </c>
       <c r="I24" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>5</v>
+        <v>128</v>
       </c>
       <c r="J24" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>5</v>
+        <v>64</v>
       </c>
       <c r="K24" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1602,37 +1839,37 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B25" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="7">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="D25" s="7">
-        <v>1</v>
+        <v>32</v>
       </c>
       <c r="E25" s="7">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G25" s="13">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="G25" s="8">
+        <v>2</v>
       </c>
       <c r="H25" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="I25" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>6</v>
+        <v>128</v>
       </c>
       <c r="J25" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>6</v>
+        <v>64</v>
       </c>
       <c r="K25" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1641,37 +1878,37 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B26" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C26" s="7">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D26" s="7">
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E26" s="7">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G26" s="13">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="G26" s="8">
+        <v>2</v>
       </c>
       <c r="H26" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="I26" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>7</v>
+        <v>128</v>
       </c>
       <c r="J26" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>7</v>
+        <v>64</v>
       </c>
       <c r="K26" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1680,37 +1917,37 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="B27" s="7">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="7">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="D27" s="7">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E27" s="7">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G27" s="13">
-        <v>8</v>
+        <v>11</v>
+      </c>
+      <c r="G27" s="8">
+        <v>2</v>
       </c>
       <c r="H27" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="I27" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>8</v>
+        <v>128</v>
       </c>
       <c r="J27" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>64</v>
       </c>
       <c r="K27" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
@@ -1718,40 +1955,430 @@
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="B28" s="15">
-        <v>2</v>
-      </c>
-      <c r="C28" s="15">
-        <v>16</v>
-      </c>
-      <c r="D28" s="15">
-        <v>1</v>
-      </c>
-      <c r="E28" s="15">
-        <v>16</v>
-      </c>
-      <c r="F28" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="G28" s="17">
-        <v>8</v>
+      <c r="A28" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B28" s="7">
+        <v>1</v>
+      </c>
+      <c r="C28" s="7">
+        <v>2</v>
+      </c>
+      <c r="D28" s="7">
+        <v>1</v>
+      </c>
+      <c r="E28" s="7">
+        <v>0</v>
+      </c>
+      <c r="F28" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G28" s="8">
+        <v>2</v>
       </c>
       <c r="H28" s="9">
         <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="I28" s="9">
         <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="J28" s="10">
         <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K28" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B29" s="7">
+        <v>1</v>
+      </c>
+      <c r="C29" s="7">
+        <v>4</v>
+      </c>
+      <c r="D29" s="7">
+        <v>1</v>
+      </c>
+      <c r="E29" s="7">
+        <v>0</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G29" s="8">
+        <v>2</v>
+      </c>
+      <c r="H29" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
+      </c>
+      <c r="I29" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
+      </c>
+      <c r="J29" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="K29" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" s="7">
+        <v>1</v>
+      </c>
+      <c r="C30" s="7">
+        <v>8</v>
+      </c>
+      <c r="D30" s="7">
+        <v>1</v>
+      </c>
+      <c r="E30" s="7">
+        <v>0</v>
+      </c>
+      <c r="F30" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G30" s="8">
+        <v>2</v>
+      </c>
+      <c r="H30" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="I30" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="J30" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="K30" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B31" s="7">
+        <v>1</v>
+      </c>
+      <c r="C31" s="7">
+        <v>16</v>
+      </c>
+      <c r="D31" s="7">
+        <v>1</v>
+      </c>
+      <c r="E31" s="7">
+        <v>0</v>
+      </c>
+      <c r="F31" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G31" s="8">
+        <v>2</v>
+      </c>
+      <c r="H31" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="I31" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="J31" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="K31" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A32" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="7">
+        <v>1</v>
+      </c>
+      <c r="C32" s="7">
+        <v>1</v>
+      </c>
+      <c r="D32" s="7">
+        <v>2</v>
+      </c>
+      <c r="E32" s="7">
+        <v>0</v>
+      </c>
+      <c r="F32" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G32" s="8">
+        <v>2</v>
+      </c>
+      <c r="H32" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>2</v>
+      </c>
+      <c r="I32" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>2</v>
+      </c>
+      <c r="J32" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>2</v>
+      </c>
+      <c r="K32" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A33" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="7">
+        <v>1</v>
+      </c>
+      <c r="C33" s="7">
+        <v>1</v>
+      </c>
+      <c r="D33" s="7">
+        <v>4</v>
+      </c>
+      <c r="E33" s="7">
+        <v>0</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G33" s="8">
+        <v>2</v>
+      </c>
+      <c r="H33" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>4</v>
+      </c>
+      <c r="I33" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>4</v>
+      </c>
+      <c r="J33" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>4</v>
+      </c>
+      <c r="K33" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A34" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B34" s="7">
+        <v>1</v>
+      </c>
+      <c r="C34" s="7">
+        <v>1</v>
+      </c>
+      <c r="D34" s="7">
+        <v>8</v>
+      </c>
+      <c r="E34" s="7">
+        <v>0</v>
+      </c>
+      <c r="F34" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G34" s="8">
+        <v>2</v>
+      </c>
+      <c r="H34" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>8</v>
+      </c>
+      <c r="I34" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>8</v>
+      </c>
+      <c r="J34" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>8</v>
+      </c>
+      <c r="K34" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A35" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B35" s="7">
+        <v>1</v>
+      </c>
+      <c r="C35" s="7">
+        <v>1</v>
+      </c>
+      <c r="D35" s="7">
+        <v>16</v>
+      </c>
+      <c r="E35" s="7">
+        <v>0</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G35" s="8">
+        <v>2</v>
+      </c>
+      <c r="H35" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>16</v>
+      </c>
+      <c r="I35" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>16</v>
+      </c>
+      <c r="J35" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>16</v>
+      </c>
+      <c r="K35" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B36" s="7">
+        <v>1</v>
+      </c>
+      <c r="C36" s="7">
+        <v>1</v>
+      </c>
+      <c r="D36" s="7">
+        <v>32</v>
+      </c>
+      <c r="E36" s="7">
+        <v>0</v>
+      </c>
+      <c r="F36" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G36" s="8">
+        <v>2</v>
+      </c>
+      <c r="H36" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>32</v>
+      </c>
+      <c r="I36" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>32</v>
+      </c>
+      <c r="J36" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>32</v>
+      </c>
+      <c r="K36" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="B37" s="7">
+        <v>1</v>
+      </c>
+      <c r="C37" s="7">
+        <v>1</v>
+      </c>
+      <c r="D37" s="7">
+        <v>64</v>
+      </c>
+      <c r="E37" s="7">
+        <v>0</v>
+      </c>
+      <c r="F37" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" s="8">
+        <v>2</v>
+      </c>
+      <c r="H37" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>64</v>
+      </c>
+      <c r="I37" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>64</v>
+      </c>
+      <c r="J37" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>64</v>
+      </c>
+      <c r="K37" t="b">
+        <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B38" s="7">
+        <v>1</v>
+      </c>
+      <c r="C38" s="7">
+        <v>1</v>
+      </c>
+      <c r="D38" s="7">
+        <v>1</v>
+      </c>
+      <c r="E38" s="7">
+        <v>0</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="G38" s="8">
+        <v>2</v>
+      </c>
+      <c r="H38" s="9">
+        <f>Table1[[#This Row], [n_mpi_procs]]*Table1[[#This Row], [n_omp_threads]]</f>
+        <v>1</v>
+      </c>
+      <c r="I38" s="9">
+        <f>Table1[[#This Row], [n_omp_threads]]*Table1[[#This Row], [n_mpi_procs]]</f>
+        <v>1</v>
+      </c>
+      <c r="J38" s="10">
+        <f>Table1[[#This Row], [total_devices]]/Table1[[#This Row], [n_nodes]]</f>
+        <v>1</v>
+      </c>
+      <c r="K38" t="b">
         <f>Table1[[#This Row], [n_mpi_procs]]&gt;=Table1[[#This Row], [n_nodes]]</f>
         <v>1</v>
       </c>

</xml_diff>